<commit_message>
Auto update portfolio 2026-08-13 13:18 UTC
</commit_message>
<xml_diff>
--- a/data/Portfolio.xlsx
+++ b/data/Portfolio.xlsx
@@ -556,34 +556,34 @@
         <v>1765.63</v>
       </c>
       <c r="J2" t="n">
-        <v>63878000</v>
+        <v>68878000</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>64274000</v>
+        <v>69274000</v>
       </c>
       <c r="M2" t="n">
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.006161122693468588</v>
+        <v>-0.005716430406790427</v>
       </c>
       <c r="O2" t="n">
         <v>-0.01536376716224808</v>
       </c>
       <c r="P2" t="n">
-        <v>0.3573945474697229</v>
+        <v>0.4636435336206453</v>
       </c>
       <c r="Q2" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R2" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S2" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="3">
@@ -617,34 +617,34 @@
         <v>1793.18</v>
       </c>
       <c r="J3" t="n">
-        <v>64274000</v>
+        <v>69274000</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>64042000</v>
+        <v>69042000</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.003622622653883389</v>
+        <v>0.003360273456736479</v>
       </c>
       <c r="O3" t="n">
         <v>0.01114801427757817</v>
       </c>
       <c r="P3" t="n">
-        <v>0.365809467172876</v>
+        <v>0.4720584533237981</v>
       </c>
       <c r="Q3" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R3" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S3" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="4">
@@ -678,34 +678,34 @@
         <v>1773.41</v>
       </c>
       <c r="J4" t="n">
-        <v>64042000</v>
+        <v>69042000</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>66099000</v>
+        <v>71099000</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.03111998668663671</v>
+        <v>-0.02893148989437264</v>
       </c>
       <c r="O4" t="n">
         <v>-0.001891072001440786</v>
       </c>
       <c r="P4" t="n">
-        <v>0.3608795142154733</v>
+        <v>0.4671285003663954</v>
       </c>
       <c r="Q4" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R4" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S4" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="5">
@@ -739,34 +739,34 @@
         <v>1776.77</v>
       </c>
       <c r="J5" t="n">
-        <v>66099000</v>
+        <v>71099000</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>65570000</v>
+        <v>70570000</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0.00806771389354888</v>
+        <v>0.007496103159982995</v>
       </c>
       <c r="O5" t="n">
         <v>0.004926303405992982</v>
       </c>
       <c r="P5" t="n">
-        <v>0.4045903471179628</v>
+        <v>0.510839333268885</v>
       </c>
       <c r="Q5" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R5" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S5" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="6">
@@ -800,34 +800,34 @@
         <v>1768.06</v>
       </c>
       <c r="J6" t="n">
-        <v>65570000</v>
+        <v>70570000</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>66134000</v>
+        <v>71134000</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>-0.008528139837300027</v>
+        <v>-0.007928697950347232</v>
       </c>
       <c r="O6" t="n">
         <v>0.001858588605945233</v>
       </c>
       <c r="P6" t="n">
-        <v>0.393349204383195</v>
+        <v>0.4995981905341174</v>
       </c>
       <c r="Q6" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R6" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S6" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="7">
@@ -861,34 +861,34 @@
         <v>1764.78</v>
       </c>
       <c r="J7" t="n">
-        <v>66134000</v>
+        <v>71134000</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>68405000</v>
+        <v>73405000</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>-0.03319932753453695</v>
+        <v>-0.03093794700633472</v>
       </c>
       <c r="O7" t="n">
         <v>-0.006574873625074584</v>
       </c>
       <c r="P7" t="n">
-        <v>0.4053340900210192</v>
+        <v>0.5115830761719413</v>
       </c>
       <c r="Q7" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R7" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S7" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="8">
@@ -922,34 +922,34 @@
         <v>1776.46</v>
       </c>
       <c r="J8" t="n">
-        <v>68405000</v>
+        <v>73405000</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>65031000</v>
+        <v>70031000</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0.05188294813242915</v>
+        <v>0.0481786637346318</v>
       </c>
       <c r="O8" t="n">
         <v>-0.0004332584977746468</v>
       </c>
       <c r="P8" t="n">
-        <v>0.4535923795307681</v>
+        <v>0.5598413656816901</v>
       </c>
       <c r="Q8" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R8" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S8" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="9">
@@ -983,34 +983,34 @@
         <v>1777.23</v>
       </c>
       <c r="J9" t="n">
-        <v>65031000</v>
+        <v>70031000</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>61637000</v>
+        <v>66637000</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0.05506432824439866</v>
+        <v>0.050932665035941</v>
       </c>
       <c r="O9" t="n">
         <v>0.008162964307594667</v>
       </c>
       <c r="P9" t="n">
-        <v>0.3818955636761256</v>
+        <v>0.4881445498270478</v>
       </c>
       <c r="Q9" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R9" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S9" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="10">
@@ -1044,34 +1044,34 @@
         <v>1762.84</v>
       </c>
       <c r="J10" t="n">
-        <v>61637000</v>
+        <v>66637000</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>55883000</v>
+        <v>60883000</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1029651235617272</v>
+        <v>0.09450914048256492</v>
       </c>
       <c r="O10" t="n">
         <v>0.01558953323577872</v>
       </c>
       <c r="P10" t="n">
-        <v>0.3097737518768797</v>
+        <v>0.4160227380278019</v>
       </c>
       <c r="Q10" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R10" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S10" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="11">
@@ -1105,34 +1105,34 @@
         <v>1735.78</v>
       </c>
       <c r="J11" t="n">
-        <v>55883000</v>
+        <v>60883000</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>58322000</v>
+        <v>63322000</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.041819553513254</v>
+        <v>-0.03851741890654117</v>
       </c>
       <c r="O11" t="n">
         <v>-0.005089816927080437</v>
       </c>
       <c r="P11" t="n">
-        <v>0.1875024186143983</v>
+        <v>0.2937514047653205</v>
       </c>
       <c r="Q11" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R11" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S11" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="12">
@@ -1166,34 +1166,34 @@
         <v>1744.66</v>
       </c>
       <c r="J12" t="n">
-        <v>58322000</v>
+        <v>63322000</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>57806000</v>
+        <v>62806000</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.00892640902328478</v>
+        <v>0.008215775562844314</v>
       </c>
       <c r="O12" t="n">
         <v>0.02345308210338604</v>
       </c>
       <c r="P12" t="n">
-        <v>0.2393306740588181</v>
+        <v>0.3455796602097403</v>
       </c>
       <c r="Q12" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R12" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S12" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="13">
@@ -1227,34 +1227,34 @@
         <v>1704.68</v>
       </c>
       <c r="J13" t="n">
-        <v>57806000</v>
+        <v>62806000</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>56530000</v>
+        <v>61530000</v>
       </c>
       <c r="M13" t="n">
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>0.02257208561825579</v>
+        <v>0.020737851454575</v>
       </c>
       <c r="O13" t="n">
         <v>0.01431614523211677</v>
       </c>
       <c r="P13" t="n">
-        <v>0.2283657786880429</v>
+        <v>0.3346147648389652</v>
       </c>
       <c r="Q13" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R13" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S13" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="14">
@@ -1288,34 +1288,34 @@
         <v>1680.62</v>
       </c>
       <c r="J14" t="n">
-        <v>56530000</v>
+        <v>61530000</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>56299000</v>
+        <v>61299000</v>
       </c>
       <c r="M14" t="n">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>0.004103092417272065</v>
+        <v>0.003768413840356286</v>
       </c>
       <c r="O14" t="n">
         <v>0.006956219555305232</v>
       </c>
       <c r="P14" t="n">
-        <v>0.2012510374223275</v>
+        <v>0.3075000235732497</v>
       </c>
       <c r="Q14" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R14" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S14" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="15">
@@ -1349,7 +1349,7 @@
         <v>1669.01</v>
       </c>
       <c r="J15" t="n">
-        <v>56299000</v>
+        <v>61299000</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1361,22 +1361,22 @@
         <v>5000000</v>
       </c>
       <c r="N15" t="n">
-        <v>-0.0355136024121154</v>
+        <v>0.05014390461180018</v>
       </c>
       <c r="O15" t="n">
         <v>-0.01014168707854168</v>
       </c>
       <c r="P15" t="n">
-        <v>0.1963423342621549</v>
+        <v>0.3025913204130772</v>
       </c>
       <c r="Q15" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R15" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S15" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="16">
@@ -1431,13 +1431,13 @@
         <v>0.2403931639203274</v>
       </c>
       <c r="Q16" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R16" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S16" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="17">
@@ -1492,13 +1492,13 @@
         <v>0.3441620966360635</v>
       </c>
       <c r="Q17" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R17" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S17" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="18">
@@ -1553,13 +1553,13 @@
         <v>0.4327317276729437</v>
       </c>
       <c r="Q18" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R18" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S18" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="19">
@@ -1614,13 +1614,13 @@
         <v>0.5560096822457936</v>
       </c>
       <c r="Q19" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R19" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S19" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="20">
@@ -1675,13 +1675,13 @@
         <v>0.7060015590179358</v>
       </c>
       <c r="Q20" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R20" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S20" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="21">
@@ -1736,13 +1736,13 @@
         <v>0.8130791703255869</v>
       </c>
       <c r="Q21" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R21" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S21" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="22">
@@ -1797,13 +1797,13 @@
         <v>0.7364881638954253</v>
       </c>
       <c r="Q22" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R22" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S22" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="23">
@@ -1858,13 +1858,13 @@
         <v>0.8465617290945857</v>
       </c>
       <c r="Q23" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R23" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S23" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="24">
@@ -1919,13 +1919,13 @@
         <v>1.032810196016754</v>
       </c>
       <c r="Q24" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R24" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S24" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="25">
@@ -1980,13 +1980,13 @@
         <v>0.8988522206269489</v>
       </c>
       <c r="Q25" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R25" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S25" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="26">
@@ -2041,13 +2041,13 @@
         <v>1.028871071455695</v>
       </c>
       <c r="Q26" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R26" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S26" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="27">
@@ -2102,13 +2102,13 @@
         <v>1.20155452492464</v>
       </c>
       <c r="Q27" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R27" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S27" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="28">
@@ -2163,13 +2163,13 @@
         <v>1.309370028579644</v>
       </c>
       <c r="Q28" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R28" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S28" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="29">
@@ -2224,13 +2224,13 @@
         <v>1.238609976999804</v>
       </c>
       <c r="Q29" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R29" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S29" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="30">
@@ -2285,13 +2285,13 @@
         <v>1.303777862881026</v>
       </c>
       <c r="Q30" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R30" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S30" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="31">
@@ -2346,13 +2346,13 @@
         <v>1.315701227540468</v>
       </c>
       <c r="Q31" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R31" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S31" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="32">
@@ -2407,13 +2407,13 @@
         <v>1.361318827382255</v>
       </c>
       <c r="Q32" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R32" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S32" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="33">
@@ -2468,13 +2468,13 @@
         <v>1.375280351392754</v>
       </c>
       <c r="Q33" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R33" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S33" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="34">
@@ -2529,13 +2529,13 @@
         <v>1.28598632617053</v>
       </c>
       <c r="Q34" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R34" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S34" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="35">
@@ -2590,13 +2590,13 @@
         <v>1.307189924132998</v>
       </c>
       <c r="Q35" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R35" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S35" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="36">
@@ -2651,13 +2651,13 @@
         <v>1.313461410854292</v>
       </c>
       <c r="Q36" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R36" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S36" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="37">
@@ -2712,13 +2712,13 @@
         <v>1.320628824250055</v>
       </c>
       <c r="Q37" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R37" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S37" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="38">
@@ -2773,13 +2773,13 @@
         <v>1.321674072036938</v>
       </c>
       <c r="Q38" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R38" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S38" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="39">
@@ -2834,13 +2834,13 @@
         <v>1.30950440137538</v>
       </c>
       <c r="Q39" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R39" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S39" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="40">
@@ -2895,13 +2895,13 @@
         <v>1.31077363083088</v>
       </c>
       <c r="Q40" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R40" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S40" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="41">
@@ -2956,13 +2956,13 @@
         <v>1.346237395028669</v>
       </c>
       <c r="Q41" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R41" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S41" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="42">
@@ -3017,13 +3017,13 @@
         <v>1.359452313477108</v>
       </c>
       <c r="Q42" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R42" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S42" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="43">
@@ -3078,13 +3078,13 @@
         <v>1.393721508775604</v>
       </c>
       <c r="Q43" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R43" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S43" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="44">
@@ -3139,13 +3139,13 @@
         <v>1.430902465766128</v>
       </c>
       <c r="Q44" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R44" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S44" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="45">
@@ -3200,13 +3200,13 @@
         <v>1.423511070701747</v>
       </c>
       <c r="Q45" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R45" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S45" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="46">
@@ -3261,13 +3261,13 @@
         <v>1.356988515122314</v>
       </c>
       <c r="Q46" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R46" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S46" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="47">
@@ -3322,13 +3322,13 @@
         <v>1.345341468354198</v>
       </c>
       <c r="Q47" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R47" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S47" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="48">
@@ -3383,13 +3383,13 @@
         <v>1.40372602330719</v>
       </c>
       <c r="Q48" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R48" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S48" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="49">
@@ -3444,13 +3444,13 @@
         <v>1.392758835563885</v>
       </c>
       <c r="Q49" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R49" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S49" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="50">
@@ -3505,13 +3505,13 @@
         <v>1.362094088762943</v>
       </c>
       <c r="Q50" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R50" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S50" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="51">
@@ -3566,13 +3566,13 @@
         <v>1.451665435591374</v>
       </c>
       <c r="Q51" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R51" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S51" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="52">
@@ -3627,13 +3627,13 @@
         <v>1.484450214269912</v>
       </c>
       <c r="Q52" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R52" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S52" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="53">
@@ -3688,13 +3688,13 @@
         <v>1.507013410681469</v>
       </c>
       <c r="Q53" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R53" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S53" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="54">
@@ -3749,13 +3749,13 @@
         <v>1.440662773008347</v>
       </c>
       <c r="Q54" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R54" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S54" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="55">
@@ -3810,13 +3810,13 @@
         <v>1.392671334574214</v>
       </c>
       <c r="Q55" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R55" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S55" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="56">
@@ -3871,13 +3871,13 @@
         <v>1.349727124068092</v>
       </c>
       <c r="Q56" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R56" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S56" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="57">
@@ -3932,13 +3932,13 @@
         <v>1.334756532756197</v>
       </c>
       <c r="Q57" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R57" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S57" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="58">
@@ -3993,13 +3993,13 @@
         <v>1.364370930741533</v>
       </c>
       <c r="Q58" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R58" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S58" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="59">
@@ -4054,13 +4054,13 @@
         <v>1.425877757451427</v>
       </c>
       <c r="Q59" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R59" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S59" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="60">
@@ -4115,13 +4115,13 @@
         <v>1.383607633773362</v>
       </c>
       <c r="Q60" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R60" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S60" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="61">
@@ -4176,13 +4176,13 @@
         <v>1.429252617625325</v>
       </c>
       <c r="Q61" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R61" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S61" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="62">
@@ -4237,13 +4237,13 @@
         <v>1.48367223792942</v>
       </c>
       <c r="Q62" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R62" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S62" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="63">
@@ -4298,13 +4298,13 @@
         <v>1.514045979494497</v>
       </c>
       <c r="Q63" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R63" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S63" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="64">
@@ -4359,13 +4359,13 @@
         <v>1.40900345658194</v>
       </c>
       <c r="Q64" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R64" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S64" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="65">
@@ -4420,13 +4420,13 @@
         <v>1.429500179870741</v>
       </c>
       <c r="Q65" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R65" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S65" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="66">
@@ -4481,13 +4481,13 @@
         <v>1.37183999321661</v>
       </c>
       <c r="Q66" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R66" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S66" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="67">
@@ -4542,13 +4542,13 @@
         <v>1.421924388918471</v>
       </c>
       <c r="Q67" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R67" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S67" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="68">
@@ -4603,13 +4603,13 @@
         <v>1.312496297469028</v>
       </c>
       <c r="Q68" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R68" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S68" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="69">
@@ -4664,13 +4664,13 @@
         <v>1.304078751972916</v>
       </c>
       <c r="Q69" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R69" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S69" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="70">
@@ -4725,13 +4725,13 @@
         <v>1.287243660980694</v>
       </c>
       <c r="Q70" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R70" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S70" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="71">
@@ -4786,13 +4786,13 @@
         <v>1.331769636043869</v>
       </c>
       <c r="Q71" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R71" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S71" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="72">
@@ -4847,13 +4847,13 @@
         <v>1.37147533871003</v>
       </c>
       <c r="Q72" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R72" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S72" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="73">
@@ -4908,13 +4908,13 @@
         <v>1.375654886363731</v>
       </c>
       <c r="Q73" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R73" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S73" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="74">
@@ -4969,13 +4969,13 @@
         <v>1.385685800732614</v>
       </c>
       <c r="Q74" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R74" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S74" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="75">
@@ -5030,13 +5030,13 @@
         <v>1.382760117375023</v>
       </c>
       <c r="Q75" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R75" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S75" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="76">
@@ -5091,13 +5091,13 @@
         <v>1.435422417811657</v>
       </c>
       <c r="Q76" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R76" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S76" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="77">
@@ -5152,13 +5152,13 @@
         <v>1.414106724777781</v>
       </c>
       <c r="Q77" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R77" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S77" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="78">
@@ -5213,13 +5213,13 @@
         <v>1.391119212682425</v>
       </c>
       <c r="Q78" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R78" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S78" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="79">
@@ -5274,13 +5274,13 @@
         <v>1.402403991347418</v>
       </c>
       <c r="Q79" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R79" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S79" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="80">
@@ -5335,13 +5335,13 @@
         <v>1.420794001023703</v>
       </c>
       <c r="Q80" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R80" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S80" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="81">
@@ -5396,13 +5396,13 @@
         <v>1.442527648822949</v>
       </c>
       <c r="Q81" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R81" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S81" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="82">
@@ -5457,13 +5457,13 @@
         <v>1.48348721582922</v>
       </c>
       <c r="Q82" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R82" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S82" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="83">
@@ -5518,13 +5518,13 @@
         <v>1.442945603588319</v>
       </c>
       <c r="Q83" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R83" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S83" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="84">
@@ -5579,13 +5579,13 @@
         <v>1.390701257917055</v>
       </c>
       <c r="Q84" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R84" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S84" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="85">
@@ -5640,13 +5640,13 @@
         <v>1.418704227196852</v>
       </c>
       <c r="Q85" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R85" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S85" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="86">
@@ -5701,13 +5701,13 @@
         <v>1.464679251387565</v>
       </c>
       <c r="Q86" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R86" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S86" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="87">
@@ -5762,13 +5762,13 @@
         <v>1.433332643984806</v>
       </c>
       <c r="Q87" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R87" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S87" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="88">
@@ -5823,13 +5823,13 @@
         <v>1.485576989656071</v>
       </c>
       <c r="Q88" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R88" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S88" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="89">
@@ -5884,13 +5884,13 @@
         <v>1.497697677851804</v>
       </c>
       <c r="Q89" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R89" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S89" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="90">
@@ -5945,13 +5945,13 @@
         <v>1.507728592220687</v>
       </c>
       <c r="Q90" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R90" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S90" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="91">
@@ -6006,13 +6006,13 @@
         <v>1.322992585927096</v>
       </c>
       <c r="Q91" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R91" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S91" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="92">
@@ -6067,13 +6067,13 @@
         <v>1.325082359753947</v>
       </c>
       <c r="Q92" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R92" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S92" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="93">
@@ -6128,13 +6128,13 @@
         <v>1.326754178815427</v>
       </c>
       <c r="Q93" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R93" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S93" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="94">
@@ -6189,13 +6189,13 @@
         <v>1.37272920300614</v>
       </c>
       <c r="Q94" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R94" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S94" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="95">
@@ -6250,13 +6250,13 @@
         <v>1.384849891201873</v>
       </c>
       <c r="Q95" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R95" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S95" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="96">
@@ -6311,13 +6311,13 @@
         <v>1.360608514810406</v>
       </c>
       <c r="Q96" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R96" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S96" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="97">
@@ -6372,13 +6372,13 @@
         <v>1.341382595603381</v>
       </c>
       <c r="Q97" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R97" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S97" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="98">
@@ -6433,13 +6433,13 @@
         <v>1.381924207844282</v>
       </c>
       <c r="Q98" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R98" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S98" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="99">
@@ -6494,13 +6494,13 @@
         <v>1.310035988200622</v>
       </c>
       <c r="Q99" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R99" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="100">
@@ -6555,13 +6555,13 @@
         <v>1.437685035676949</v>
       </c>
       <c r="Q100" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R100" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S100" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="101">
@@ -6616,13 +6616,13 @@
         <v>1.35121310028976</v>
       </c>
       <c r="Q101" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R101" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S101" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="102">
@@ -6677,13 +6677,13 @@
         <v>1.237681919815424</v>
       </c>
       <c r="Q102" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R102" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S102" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="103">
@@ -6738,13 +6738,13 @@
         <v>1.320624388452115</v>
       </c>
       <c r="Q103" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R103" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S103" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="104">
@@ -6799,13 +6799,13 @@
         <v>1.438273280135366</v>
       </c>
       <c r="Q104" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R104" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S104" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="105">
@@ -6860,13 +6860,13 @@
         <v>1.509450859603732</v>
       </c>
       <c r="Q105" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R105" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="106">
@@ -6921,13 +6921,13 @@
         <v>1.542392549275043</v>
       </c>
       <c r="Q106" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R106" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S106" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="107">
@@ -6982,13 +6982,13 @@
         <v>1.491803525851245</v>
       </c>
       <c r="Q107" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R107" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S107" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="108">
@@ -7043,13 +7043,13 @@
         <v>1.44239099134428</v>
       </c>
       <c r="Q108" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R108" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S108" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="109">
@@ -7104,13 +7104,13 @@
         <v>1.474156192098757</v>
       </c>
       <c r="Q109" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R109" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S109" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="110">
@@ -7165,13 +7165,13 @@
         <v>1.603569972950333</v>
       </c>
       <c r="Q110" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R110" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S110" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="111">
@@ -7226,13 +7226,13 @@
         <v>1.5553339273602</v>
       </c>
       <c r="Q111" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R111" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S111" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="112">
@@ -7287,13 +7287,13 @@
         <v>1.333565766537273</v>
       </c>
       <c r="Q112" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R112" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S112" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="113">
@@ -7348,13 +7348,13 @@
         <v>1.650041285165217</v>
       </c>
       <c r="Q113" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R113" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S113" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="114">
@@ -7409,13 +7409,13 @@
         <v>1.757690021055391</v>
       </c>
       <c r="Q114" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R114" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S114" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="115">
@@ -7470,13 +7470,13 @@
         <v>1.807102555562357</v>
       </c>
       <c r="Q115" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R115" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S115" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="116">
@@ -7531,13 +7531,13 @@
         <v>1.887103801906967</v>
       </c>
       <c r="Q116" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R116" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S116" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="117">
@@ -7592,13 +7592,13 @@
         <v>2.028870716385283</v>
       </c>
       <c r="Q117" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R117" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S117" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="118">
@@ -7653,13 +7653,13 @@
         <v>2.136735021298073</v>
       </c>
       <c r="Q118" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R118" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S118" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="119">
@@ -7714,13 +7714,13 @@
         <v>2.114397728518159</v>
       </c>
       <c r="Q119" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R119" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S119" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="120">
@@ -7775,13 +7775,13 @@
         <v>2.073446025088314</v>
       </c>
       <c r="Q120" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R120" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S120" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="121">
@@ -7836,13 +7836,13 @@
         <v>2.123084453488125</v>
       </c>
       <c r="Q121" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R121" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S121" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="122">
@@ -7897,13 +7897,13 @@
         <v>2.125859241635675</v>
       </c>
       <c r="Q122" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R122" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S122" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="123">
@@ -7958,13 +7958,13 @@
         <v>2.088909141925205</v>
       </c>
       <c r="Q123" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R123" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S123" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="124">
@@ -8019,13 +8019,13 @@
         <v>2.085333325824192</v>
       </c>
       <c r="Q124" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R124" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S124" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="125">
@@ -8080,13 +8080,13 @@
         <v>2.078777662972335</v>
       </c>
       <c r="Q125" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R125" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S125" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="126">
@@ -8141,13 +8141,13 @@
         <v>2.022756544056462</v>
       </c>
       <c r="Q126" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R126" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S126" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="127">
@@ -8202,13 +8202,13 @@
         <v>2.036463839110346</v>
       </c>
       <c r="Q127" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R127" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S127" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="128">
@@ -8263,13 +8263,13 @@
         <v>1.977462873443629</v>
       </c>
       <c r="Q128" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R128" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S128" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="129">
@@ -8324,13 +8324,13 @@
         <v>2.147314138241755</v>
       </c>
       <c r="Q129" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R129" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S129" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="130">
@@ -8385,13 +8385,13 @@
         <v>2.272467701777216</v>
       </c>
       <c r="Q130" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R130" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S130" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="131">
@@ -8446,13 +8446,13 @@
         <v>2.213466736110498</v>
       </c>
       <c r="Q131" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R131" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S131" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="132">
@@ -8507,13 +8507,13 @@
         <v>2.230153877915226</v>
       </c>
       <c r="Q132" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R132" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S132" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="133">
@@ -8568,13 +8568,13 @@
         <v>2.188436023403406</v>
       </c>
       <c r="Q133" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R133" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S133" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="134">
@@ -8629,13 +8629,13 @@
         <v>2.151485923692937</v>
       </c>
       <c r="Q134" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R134" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S134" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="135">
@@ -8690,13 +8690,13 @@
         <v>2.052555011564906</v>
       </c>
       <c r="Q135" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R135" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S135" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="136">
@@ -8751,13 +8751,13 @@
         <v>1.950644252686031</v>
       </c>
       <c r="Q136" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R136" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S136" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="137">
@@ -8812,13 +8812,13 @@
         <v>1.794500282941789</v>
       </c>
       <c r="Q137" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R137" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S137" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="138">
@@ -8873,13 +8873,13 @@
         <v>1.935745018931809</v>
       </c>
       <c r="Q138" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R138" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="139">
@@ -8934,13 +8934,13 @@
         <v>2.006493656695451</v>
       </c>
       <c r="Q139" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R139" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S139" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="140">
@@ -8995,13 +8995,13 @@
         <v>2.004242628265444</v>
       </c>
       <c r="Q140" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R140" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S140" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="141">
@@ -9056,13 +9056,13 @@
         <v>2.024292562818765</v>
       </c>
       <c r="Q141" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R141" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S141" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="142">
@@ -9117,13 +9117,13 @@
         <v>2.0764223926574</v>
       </c>
       <c r="Q142" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R142" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S142" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="143">
@@ -9178,13 +9178,13 @@
         <v>2.083551258276358</v>
       </c>
       <c r="Q143" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R143" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S143" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="144">
@@ -9239,13 +9239,13 @@
         <v>1.887507453754997</v>
       </c>
       <c r="Q144" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R144" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S144" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="145">
@@ -9300,13 +9300,13 @@
         <v>1.92136956544505</v>
       </c>
       <c r="Q145" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R145" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S145" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="146">
@@ -9361,13 +9361,13 @@
         <v>1.936963958986522</v>
       </c>
       <c r="Q146" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R146" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S146" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="147">
@@ -9422,13 +9422,13 @@
         <v>1.967707191968281</v>
       </c>
       <c r="Q147" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R147" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S147" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="148">
@@ -9483,13 +9483,13 @@
         <v>1.850526463356649</v>
       </c>
       <c r="Q148" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R148" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S148" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="149">
@@ -9544,13 +9544,13 @@
         <v>1.892854102969216</v>
       </c>
       <c r="Q149" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R149" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S149" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="150">
@@ -9605,13 +9605,13 @@
         <v>2.012262602086772</v>
       </c>
       <c r="Q150" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R150" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S150" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="151">
@@ -9666,13 +9666,13 @@
         <v>1.934736188480598</v>
       </c>
       <c r="Q151" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R151" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S151" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="152">
@@ -9727,13 +9727,13 @@
         <v>1.915577362129647</v>
       </c>
       <c r="Q152" t="n">
-        <v>-1.066479692960254</v>
+        <v>-1.002788071077717</v>
       </c>
       <c r="R152" t="n">
-        <v>-0.6371232577881553</v>
+        <v>-0.6209609148329583</v>
       </c>
       <c r="S152" t="n">
-        <v>-0.5357815878530054</v>
+        <v>-0.4994452582757648</v>
       </c>
     </row>
     <row r="153">

</xml_diff>